<commit_message>
Glider Design Sensitivity Analysis
- Python
- Refactored workflow robust post-check to evaluate only kept candidates,
- Expanded RobustSummary with thesis-grade statistics: success/failure counts, failure rate, median/p90/p95 sink metrics, tail-risk, percentile margins, control/roll diagnostics, structural proxy extremes, and worst-case scenario IDs/tags
- Added RobustDrivers workbook output to rank dominant uncertainty drivers for key robust outputs using per-candidate Spearman correlations
- Enriched RobustSummaryByTag and console reporting with failure-rate and percentile-based robustness diagnostics
- Updated F_analysis consumers to read the new robust schema and keep figures and tables aligned with the revised workbook outputs.
</commit_message>
<xml_diff>
--- a/02_Glider_Design/C_results/main_text_tables.xlsx
+++ b/02_Glider_Design/C_results/main_text_tables.xlsx
@@ -2734,7 +2734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U10"/>
+  <dimension ref="A1:AF10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2750,95 +2750,150 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>robust_rank</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>selected_flag</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>objective</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>n_success</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>n_total</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>nom_success_rate</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>nom_failure_rate</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>nom_sink_mean</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>nom_sink_tail_mean_k</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>nom_sink_p95</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>nom_sink_worst</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>nom_resid_rmse_success_only</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>nom_roll_tau_p95</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>nom_roll_tau_worst</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>nom_delta_e_util_p95</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>nom_delta_e_util_worst</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>nom_alpha_worst</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>nom_alpha_p95</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>nom_alpha_margin_p05</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>nom_alpha_margin_worst</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>nom_cl_margin_p05</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>nom_cl_margin_worst</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>nom_wing_deflection_over_allow_worst</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>nom_htail_deflection_over_allow_worst</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>wing_span_m</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>wing_chord_m</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>boom_length_m</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>mass_total_kg</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>static_margin</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>L_over_D</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>sink_rate_mps</t>
         </is>
@@ -2853,61 +2908,70 @@
       <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="b">
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="b">
         <v>1</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>2.166267395066876</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="n">
         <v>1</v>
       </c>
-      <c r="F2" t="n">
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="n">
         <v>0.7162069461328315</v>
       </c>
-      <c r="G2" t="n">
+      <c r="K2" t="n">
         <v>0.7162069461328315</v>
       </c>
-      <c r="H2" t="n">
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="n">
         <v>0.7162069461328315</v>
       </c>
-      <c r="I2" t="n">
+      <c r="N2" t="n">
         <v>1.4285713188503e-17</v>
       </c>
-      <c r="J2" t="n">
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="n">
         <v>0.02553436812845662</v>
       </c>
-      <c r="K2" t="n">
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="n">
         <v>0.01588149296636211</v>
       </c>
-      <c r="L2" t="n">
-        <v>4.886000453231397</v>
-      </c>
-      <c r="M2" t="n">
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="n">
         <v>3.113999546768603</v>
       </c>
-      <c r="N2" t="n">
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="n">
         <v>0.8402748655179237</v>
       </c>
-      <c r="O2" t="n">
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="n">
         <v>0.761569966525819</v>
       </c>
-      <c r="P2" t="n">
+      <c r="AA2" t="n">
         <v>0.1646396706102183</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="AB2" t="n">
         <v>0.5639716234248189</v>
       </c>
-      <c r="R2" t="n">
+      <c r="AC2" t="n">
         <v>0.1175251467546148</v>
       </c>
-      <c r="S2" t="n">
+      <c r="AD2" t="n">
         <v>0.1000000099082708</v>
       </c>
-      <c r="T2" t="n">
+      <c r="AE2" t="n">
         <v>9.696954368874374</v>
       </c>
-      <c r="U2" t="n">
+      <c r="AF2" t="n">
         <v>0.6703135537634592</v>
       </c>
     </row>
@@ -2920,61 +2984,70 @@
       <c r="B3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="b">
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="b">
         <v>1</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>2.166267395066876</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="n">
         <v>1</v>
       </c>
-      <c r="F3" t="n">
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="n">
         <v>0.7162069461328315</v>
       </c>
-      <c r="G3" t="n">
+      <c r="K3" t="n">
         <v>0.7162069461328315</v>
       </c>
-      <c r="H3" t="n">
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="n">
         <v>0.7162069461328315</v>
       </c>
-      <c r="I3" t="n">
+      <c r="N3" t="n">
         <v>1.4285713188503e-17</v>
       </c>
-      <c r="J3" t="n">
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="n">
         <v>0.02553436812845662</v>
       </c>
-      <c r="K3" t="n">
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="n">
         <v>0.01588149296636211</v>
       </c>
-      <c r="L3" t="n">
-        <v>4.886000453231397</v>
-      </c>
-      <c r="M3" t="n">
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="n">
         <v>3.113999546768603</v>
       </c>
-      <c r="N3" t="n">
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="n">
         <v>0.8402748655179237</v>
       </c>
-      <c r="O3" t="n">
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="n">
         <v>0.761569966525819</v>
       </c>
-      <c r="P3" t="n">
+      <c r="AA3" t="n">
         <v>0.1646396706102183</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="AB3" t="n">
         <v>0.5639716234248189</v>
       </c>
-      <c r="R3" t="n">
+      <c r="AC3" t="n">
         <v>0.1175251467546148</v>
       </c>
-      <c r="S3" t="n">
+      <c r="AD3" t="n">
         <v>0.1000000099082708</v>
       </c>
-      <c r="T3" t="n">
+      <c r="AE3" t="n">
         <v>9.696954368874374</v>
       </c>
-      <c r="U3" t="n">
+      <c r="AF3" t="n">
         <v>0.6703135537634592</v>
       </c>
     </row>
@@ -2987,61 +3060,70 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="b">
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="b">
         <v>1</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>2.166267395066876</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="n">
         <v>1</v>
       </c>
-      <c r="F4" t="n">
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="n">
         <v>0.7162069461328315</v>
       </c>
-      <c r="G4" t="n">
+      <c r="K4" t="n">
         <v>0.7162069461328315</v>
       </c>
-      <c r="H4" t="n">
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="n">
         <v>0.7162069461328315</v>
       </c>
-      <c r="I4" t="n">
+      <c r="N4" t="n">
         <v>1.4285713188503e-17</v>
       </c>
-      <c r="J4" t="n">
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="n">
         <v>0.02553436812845662</v>
       </c>
-      <c r="K4" t="n">
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="n">
         <v>0.01588149296636211</v>
       </c>
-      <c r="L4" t="n">
-        <v>4.886000453231397</v>
-      </c>
-      <c r="M4" t="n">
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="n">
         <v>3.113999546768603</v>
       </c>
-      <c r="N4" t="n">
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="n">
         <v>0.8402748655179237</v>
       </c>
-      <c r="O4" t="n">
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="n">
         <v>0.761569966525819</v>
       </c>
-      <c r="P4" t="n">
+      <c r="AA4" t="n">
         <v>0.1646396706102183</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="AB4" t="n">
         <v>0.5639716234248189</v>
       </c>
-      <c r="R4" t="n">
+      <c r="AC4" t="n">
         <v>0.1175251467546148</v>
       </c>
-      <c r="S4" t="n">
+      <c r="AD4" t="n">
         <v>0.1000000099082708</v>
       </c>
-      <c r="T4" t="n">
+      <c r="AE4" t="n">
         <v>9.696954368874374</v>
       </c>
-      <c r="U4" t="n">
+      <c r="AF4" t="n">
         <v>0.6703135537634592</v>
       </c>
     </row>
@@ -3067,27 +3149,57 @@
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
+          <t>n_fail</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>failure_rate</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
           <t>success_rate</t>
         </is>
       </c>
-      <c r="C9" s="1" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>sink_mean</t>
         </is>
       </c>
-      <c r="D9" s="1" t="inlineStr">
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>sink_p95</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="inlineStr">
         <is>
           <t>sink_worst</t>
         </is>
       </c>
-      <c r="E9" s="1" t="inlineStr">
+      <c r="H9" s="1" t="inlineStr">
         <is>
           <t>nom_sink_tail_mean_k</t>
         </is>
       </c>
-      <c r="F9" s="1" t="inlineStr">
+      <c r="I9" s="1" t="inlineStr">
         <is>
           <t>nom_resid_rmse_success_only</t>
+        </is>
+      </c>
+      <c r="J9" s="1" t="inlineStr">
+        <is>
+          <t>nom_alpha_margin_worst</t>
+        </is>
+      </c>
+      <c r="K9" s="1" t="inlineStr">
+        <is>
+          <t>nom_cl_margin_worst</t>
+        </is>
+      </c>
+      <c r="L9" s="1" t="inlineStr">
+        <is>
+          <t>nom_delta_e_util_worst</t>
         </is>
       </c>
     </row>
@@ -3097,21 +3209,27 @@
           <t>mixed</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="n">
         <v>1</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0.7162069461328315</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0.7162069461328315</v>
       </c>
       <c r="E10" t="n">
         <v>0.7162069461328315</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="n">
+        <v>0.7162069461328315</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.7162069461328315</v>
+      </c>
+      <c r="I10" t="n">
         <v>1.4285713188503e-17</v>
       </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>